<commit_message>
Correcion de Loader Tables mRoyA
</commit_message>
<xml_diff>
--- a/app/database/MRA11/mroy_MRA1_02_plunger.xlsx
+++ b/app/database/MRA11/mroy_MRA1_02_plunger.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="31">
   <si>
     <t xml:space="preserve">code</t>
   </si>
@@ -58,6 +58,9 @@
     <t xml:space="preserve">H</t>
   </si>
   <si>
+    <t xml:space="preserve">3/8"</t>
+  </si>
+  <si>
     <t xml:space="preserve">metallic</t>
   </si>
   <si>
@@ -79,6 +82,9 @@
     <t xml:space="preserve">D</t>
   </si>
   <si>
+    <t xml:space="preserve">7/16"</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metallic performance limits for plunger D</t>
   </si>
   <si>
@@ -88,6 +94,9 @@
     <t xml:space="preserve">E</t>
   </si>
   <si>
+    <t xml:space="preserve">5/8"</t>
+  </si>
+  <si>
     <t xml:space="preserve">Metallic performance limits for plunger E</t>
   </si>
   <si>
@@ -97,7 +106,7 @@
     <t xml:space="preserve">F</t>
   </si>
   <si>
-    <t xml:space="preserve">1-1/16</t>
+    <t xml:space="preserve">1-1/16"</t>
   </si>
   <si>
     <t xml:space="preserve">Metallic performance limits for plunger F</t>
@@ -110,10 +119,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
-    <numFmt numFmtId="165" formatCode="mm/dd/yy"/>
-    <numFmt numFmtId="166" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
+    <numFmt numFmtId="165" formatCode="&quot;TRUE&quot;;&quot;TRUE&quot;;&quot;FALSE&quot;"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -196,7 +204,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -217,11 +225,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -230,10 +238,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -432,7 +436,7 @@
   <dimension ref="A1:K1048576"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.19"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.03"/>
@@ -444,7 +448,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="16.09"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="41.83"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="6.53"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="1" width="10.16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -482,15 +486,15 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="5" t="n">
-        <v>45724</v>
+      <c r="B2" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>9.5</v>
@@ -510,22 +514,23 @@
       <c r="I2" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J2" s="6" t="b">
+      <c r="J2" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K2" s="7" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>13</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="5" t="n">
-        <v>45724</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>12</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>9.5</v>
@@ -545,22 +550,23 @@
       <c r="I3" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J3" s="6" t="b">
+      <c r="J3" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K3" s="7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="5" t="n">
-        <v>45724</v>
+      <c r="B4" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>9.5</v>
@@ -580,22 +586,23 @@
       <c r="I4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J4" s="6" t="b">
+      <c r="J4" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K4" s="7" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>45854</v>
+        <v>19</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" s="4" t="n">
         <v>11.1</v>
@@ -615,22 +622,23 @@
       <c r="I5" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="6" t="b">
+      <c r="J5" s="6" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K5" s="7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>45854</v>
+      <c r="B6" s="5" t="s">
+        <v>20</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="4" t="n">
         <v>11.1</v>
@@ -650,22 +658,23 @@
       <c r="I6" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J6" s="9" t="b">
+      <c r="J6" s="8" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K6" s="7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>45785</v>
+        <v>23</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D7" s="4" t="n">
         <v>15.9</v>
@@ -685,22 +694,23 @@
       <c r="I7" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="9" t="b">
+      <c r="J7" s="8" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K7" s="7" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>45785</v>
+        <v>23</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>24</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D8" s="4" t="n">
         <v>15.9</v>
@@ -720,22 +730,23 @@
       <c r="I8" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="9" t="b">
+      <c r="J8" s="8" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" s="4" t="n">
         <v>27</v>
@@ -755,22 +766,23 @@
       <c r="I9" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J9" s="9" t="b">
+      <c r="J9" s="8" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K9" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>25</v>
+        <v>27</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>28</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>27</v>
@@ -790,11 +802,12 @@
       <c r="I10" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="J10" s="9" t="b">
+      <c r="J10" s="8" t="n">
+        <f aca="false">FALSE()</f>
         <v>0</v>
       </c>
       <c r="K10" s="7" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>